<commit_message>
pb đang làm thuật toán
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>/static/images/dai-noi-hue.png</t>
+          <t>/static/images/hoang-thanh-hue.png</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1574,31 +1574,31 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Đồi Vọng Cảnh</t>
+          <t>Ga Huế</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Đồi cao ngắm toàn cảnh Huế và sông Hương lúc hoàng hôn.</t>
+          <t>Nhà ga cổ kính xây dựng từ thời Pháp thuộc, điểm check-in hoài cổ và là đầu mối giao thông quan trọng.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Thiên nhiên</t>
+          <t>Tham quan</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>4.7</v>
+        <v>4.6</v>
       </c>
       <c r="F30" t="n">
-        <v>16.42723</v>
+        <v>16.45648</v>
       </c>
       <c r="G30" t="n">
-        <v>107.56493</v>
+        <v>107.57805</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>/static/images/doi-vong-canh.png</t>
+          <t>/static/images/ga-hue.png</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1613,31 +1613,31 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Núi Ngự Bình</t>
+          <t>Cầu Gỗ Lim</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ngọn núi bình phong trấn giữ Huế.</t>
+          <t>Tuyến đường đi bộ lát gỗ lim bên bờ sông Hương, điểm ngắm hoàng hôn và check-in cực hot.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Thiên nhiên</t>
+          <t>Tham quan</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="F31" t="n">
-        <v>16.44168</v>
+        <v>16.46561</v>
       </c>
       <c r="G31" t="n">
-        <v>107.5961</v>
+        <v>107.58744</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>/static/images/nui-ngu-binh.png</t>
+          <t>/static/images/cau-go-lim.png</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1652,12 +1652,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Đầm Lập An</t>
+          <t>Đồi Vọng Cảnh</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tuyệt tình cốc của Huế, vẻ đẹp mơ màng giữa đầm nước và núi Bạch Mã.</t>
+          <t>Đồi cao ngắm toàn cảnh Huế và sông Hương lúc hoàng hôn.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1669,14 +1669,14 @@
         <v>4.7</v>
       </c>
       <c r="F32" t="n">
-        <v>16.22142</v>
+        <v>16.42723</v>
       </c>
       <c r="G32" t="n">
-        <v>108.06157</v>
+        <v>107.56493</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>/static/images/dam-lap-an.png</t>
+          <t>/static/images/doi-vong-canh.png</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Vườn Quốc gia Bạch Mã</t>
+          <t>Núi Ngự Bình</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Thiên đường trên mặt đất với khí hậu mát mẻ.</t>
+          <t>Ngọn núi bình phong trấn giữ Huế.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1705,17 +1705,17 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="F33" t="n">
-        <v>16.2165</v>
+        <v>16.44168</v>
       </c>
       <c r="G33" t="n">
-        <v>107.89365</v>
+        <v>107.5961</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>/static/images/vuon-quoc-gia-bach-ma.png</t>
+          <t>/static/images/nui-ngu-binh.png</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1730,12 +1730,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Rừng ngập mặn Rú Chá</t>
+          <t>Đầm Lập An</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Khu rừng ngập mặn nguyên sinh duy nhất còn lại ở phá Tam Giang.</t>
+          <t>Tuyệt tình cốc của Huế, vẻ đẹp mơ màng giữa đầm nước và núi Bạch Mã.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1744,17 +1744,17 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="F34" t="n">
-        <v>16.55748</v>
+        <v>16.22142</v>
       </c>
       <c r="G34" t="n">
-        <v>107.61144</v>
+        <v>108.06157</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>/static/images/rung-ru-cha.png</t>
+          <t>/static/images/dam-lap-an.png</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1769,12 +1769,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Phá Tam Giang</t>
+          <t>Vườn Quốc gia Bạch Mã</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Vùng đầm phá nước lợ lớn nhất Đông Nam Á, nơi ngắm hoàng hôn đẹp nhất.</t>
+          <t>Thiên đường trên mặt đất với khí hậu mát mẻ.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1783,17 +1783,17 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="F35" t="n">
-        <v>16.59788</v>
+        <v>16.2165</v>
       </c>
       <c r="G35" t="n">
-        <v>107.54309</v>
+        <v>107.89365</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>/static/images/pha-tam-giang.png</t>
+          <t>/static/images/vuon-quoc-gia-bach-ma.png</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1808,12 +1808,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Suối Voi</t>
+          <t>Rừng ngập mặn Rú Chá</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Dòng suối mát lạnh với tảng đá hình con voi độc đáo.</t>
+          <t>Khu rừng ngập mặn nguyên sinh duy nhất còn lại ở phá Tam Giang.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1822,17 +1822,17 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="F36" t="n">
-        <v>16.24387</v>
+        <v>16.55748</v>
       </c>
       <c r="G36" t="n">
-        <v>107.98943</v>
+        <v>107.61144</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>/static/images/suoi-voi.png</t>
+          <t>/static/images/rung-ru-cha.png</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -1847,31 +1847,31 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Bãi biển Lăng Cô</t>
+          <t>Phá Tam Giang</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Một trong những bãi biển đẹp nhất Việt Nam, vịnh Lăng Cô yên bình.</t>
+          <t>Vùng đầm phá nước lợ lớn nhất Đông Nam Á, nơi ngắm hoàng hôn đẹp nhất.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Bãi biển</t>
+          <t>Thiên nhiên</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="F37" t="n">
-        <v>16.26424</v>
+        <v>16.59788</v>
       </c>
       <c r="G37" t="n">
-        <v>108.06582</v>
+        <v>107.54309</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>/static/images/bai-bien-lang-co.png</t>
+          <t>/static/images/pha-tam-giang.png</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -1886,34 +1886,112 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>Suối Voi</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Dòng suối mát lạnh với tảng đá hình con voi độc đáo.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Thiên nhiên</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F38" t="n">
+        <v>16.24387</v>
+      </c>
+      <c r="G38" t="n">
+        <v>107.98943</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>/static/images/suoi-voi.png</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Huế</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bãi biển Lăng Cô</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Một trong những bãi biển đẹp nhất Việt Nam, vịnh Lăng Cô yên bình.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Bãi biển</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F39" t="n">
+        <v>16.26424</v>
+      </c>
+      <c r="G39" t="n">
+        <v>108.06582</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>/static/images/bai-bien-lang-co.png</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Huế</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>Bãi biển Thuận An</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Bãi biển gần trung tâm Huế, hải sản tươi và không khí địa phương.</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Bãi biển</t>
         </is>
       </c>
-      <c r="E38" t="n">
+      <c r="E40" t="n">
         <v>4.6</v>
       </c>
-      <c r="F38" t="n">
+      <c r="F40" t="n">
         <v>16.55966</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G40" t="n">
         <v>107.65428</v>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>/static/images/bai-bien-thuan-an.png</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>Huế</t>
         </is>
@@ -1930,7 +2008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1962,13 +2040,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KhachTayBalo</t>
+          <t>SinhVienHue</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1978,51 +2056,161 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KhachTayBalo</t>
+          <t>SinhVienHue</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HoiYeuThienNhien</t>
+          <t>KhachTayBalo</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HoiYeuThienNhien</t>
+          <t>KhachTayBalo</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>YeuTamLinh</t>
+          <t>KhachTayBalo</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>KhachTayBalo</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HoiYeuThienNhien</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HoiYeuThienNhien</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>HoiYeuThienNhien</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>YeuTamLinh</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>YeuTamLinh</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>YeuTamLinh</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>YeuTamLinh</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>HuongDanVien</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HuongDanVien</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HuongDanVien</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HuongDanVien</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ghi chú trong file .md
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -2008,7 +2008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2136,11 +2136,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>YeuTamLinh</t>
+          <t>HoiYeuThienNhien</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -2170,17 +2170,17 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HuongDanVien</t>
+          <t>YeuTamLinh</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18">
@@ -2190,7 +2190,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -2200,7 +2200,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -2210,6 +2210,16 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HuongDanVien</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
tiếp tục thêm địa điểm cùng danh mục phía dưới địa điểm
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Khóa luận\Khoa_luan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0D8258-1996-46A6-B1DC-B24F51246087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F00694-8A12-4C12-8E15-FEF2A7FD958F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="332">
   <si>
     <t>id</t>
   </si>
@@ -330,12 +330,6 @@
     <t>/static/images/tu-cam-thanh.png</t>
   </si>
   <si>
-    <t>Văn Miếu Huế</t>
-  </si>
-  <si>
-    <t>/static/images/van-mieu-hue.png</t>
-  </si>
-  <si>
     <t>Tượng đài Quan Thế Âm Bồ Tát</t>
   </si>
   <si>
@@ -447,12 +441,6 @@
     <t>/static/images/an-xa-tac.png</t>
   </si>
   <si>
-    <t>Bia Tiên động phương tung</t>
-  </si>
-  <si>
-    <t>/static/images/bia-tien-ong-phuong-tung.png</t>
-  </si>
-  <si>
     <t>Hồ Sơn Thọ</t>
   </si>
   <si>
@@ -507,12 +495,6 @@
     <t>/static/images/cong-vien-ho-thuy-tien.png</t>
   </si>
   <si>
-    <t>Di tích xe ô tô Thích Quảng Đức</t>
-  </si>
-  <si>
-    <t>/static/images/di-tich-xe-o-to-thich-quang-uc.png</t>
-  </si>
-  <si>
     <t>Quan Tượng Đài (Nam Đài)</t>
   </si>
   <si>
@@ -642,9 +624,6 @@
     <t>Điện Thái Hòa</t>
   </si>
   <si>
-    <t>/static/images/ien-thai-hoa.png</t>
-  </si>
-  <si>
     <t>Tây Khuyết Đài</t>
   </si>
   <si>
@@ -867,9 +846,6 @@
     <t>Tử Cấm Thành là cung điện cổ kính, biểu tượng quyền lực triều đại Minh - Thanh, nổi bật với kiến trúc nguy nga giữa lòng Bắc Kinh.</t>
   </si>
   <si>
-    <t>Văn Miếu Huế là di tích lịch sử nổi bật, lưu giữ giá trị văn hóa và truyền thống hiếu học của vùng đất cố đô.</t>
-  </si>
-  <si>
     <t>Tượng đài Quan Thế Âm Bồ Tát uy nghi giữa thiên nhiên, là điểm đến tâm linh nổi bật thu hút du khách thập phương.</t>
   </si>
   <si>
@@ -924,9 +900,6 @@
     <t>Đàn Xã Tắc là di tích lịch sử linh thiêng, nơi triều đình xưa tế lễ cầu cho quốc thái dân an tại Huế.</t>
   </si>
   <si>
-    <t>Bia Tiên động phương tung là điểm đến kỳ bí, hòa quyện giữa thiên nhiên hùng vĩ và dấu ấn lịch sử độc đáo.</t>
-  </si>
-  <si>
     <t>Hồ Sơn Thọ là điểm đến lý tưởng với cảnh sắc hữu tình, không khí trong lành, thích hợp dã ngoại và thư giãn cuối tuần.</t>
   </si>
   <si>
@@ -954,9 +927,6 @@
     <t>Công viên Hồ Thủy Tiên là điểm check-in huyền bí với hồ nước, rừng cây và rồng khổng lồ bỏ hoang giữa lòng Huế.</t>
   </si>
   <si>
-    <t>Di tích xe ô tô Thích Quảng Đức lưu giữ chiếc xe lịch sử gắn liền sự kiện tự thiêu vì hòa bình, thu hút nhiều du khách tham quan.</t>
-  </si>
-  <si>
     <t>Quan Tượng Đài (Nam Đài) là điểm ngắm cảnh lý tưởng, nơi du khách chiêm ngưỡng toàn cảnh thành phố Huế và sông Hương thơ mộng.</t>
   </si>
   <si>
@@ -1051,6 +1021,18 @@
   </si>
   <si>
     <t>Hồ Nội Kim Thủy xanh biếc, yên bình giữa núi non, là điểm đến lý tưởng để thư giãn và tận hưởng không khí trong lành.</t>
+  </si>
+  <si>
+    <t>Văn Thánh Huế</t>
+  </si>
+  <si>
+    <t>/static/images/dien-thai-hoa.png</t>
+  </si>
+  <si>
+    <t>Văn Thánh Huế là di tích lịch sử nổi bật, lưu giữ giá trị văn hóa và truyền thống hiếu học của vùng đất cố đô.</t>
+  </si>
+  <si>
+    <t>/static/images/van-thanh-hue.png</t>
   </si>
 </sst>
 </file>
@@ -1149,7 +1131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1161,6 +1143,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1376,7 +1359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1000"/>
+  <dimension ref="A1:H998"/>
   <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7.375" customWidth="1"/>
@@ -1418,14 +1401,14 @@
     </row>
     <row r="2" spans="1:8" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <f t="shared" ref="A2:A103" si="0">ROW()-ROW($A$2)+1</f>
+        <f t="shared" ref="A2:A101" si="0">ROW()-ROW($A$2)+1</f>
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>9</v>
@@ -1452,7 +1435,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>9</v>
@@ -1479,7 +1462,7 @@
         <v>14</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>9</v>
@@ -1506,7 +1489,7 @@
         <v>16</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>17</v>
@@ -1533,7 +1516,7 @@
         <v>19</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>17</v>
@@ -1560,7 +1543,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>17</v>
@@ -1587,7 +1570,7 @@
         <v>23</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>17</v>
@@ -1614,7 +1597,7 @@
         <v>25</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>17</v>
@@ -1641,7 +1624,7 @@
         <v>27</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>17</v>
@@ -1668,7 +1651,7 @@
         <v>29</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>17</v>
@@ -1695,7 +1678,7 @@
         <v>31</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>32</v>
@@ -1722,7 +1705,7 @@
         <v>34</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>32</v>
@@ -1749,7 +1732,7 @@
         <v>36</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>32</v>
@@ -1776,7 +1759,7 @@
         <v>38</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>32</v>
@@ -1803,7 +1786,7 @@
         <v>40</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>41</v>
@@ -1830,7 +1813,7 @@
         <v>43</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>41</v>
@@ -1857,7 +1840,7 @@
         <v>45</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>41</v>
@@ -1884,7 +1867,7 @@
         <v>47</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>48</v>
@@ -1911,7 +1894,7 @@
         <v>50</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>48</v>
@@ -1938,7 +1921,7 @@
         <v>52</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>48</v>
@@ -1965,7 +1948,7 @@
         <v>54</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>48</v>
@@ -1992,7 +1975,7 @@
         <v>56</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>48</v>
@@ -2019,7 +2002,7 @@
         <v>58</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>59</v>
@@ -2046,7 +2029,7 @@
         <v>61</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>59</v>
@@ -2073,7 +2056,7 @@
         <v>63</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>59</v>
@@ -2100,7 +2083,7 @@
         <v>65</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>59</v>
@@ -2127,7 +2110,7 @@
         <v>67</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>59</v>
@@ -2154,7 +2137,7 @@
         <v>69</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>59</v>
@@ -2181,7 +2164,7 @@
         <v>71</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>59</v>
@@ -2208,7 +2191,7 @@
         <v>73</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>59</v>
@@ -2235,7 +2218,7 @@
         <v>75</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>76</v>
@@ -2262,7 +2245,7 @@
         <v>78</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>76</v>
@@ -2289,7 +2272,7 @@
         <v>80</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>76</v>
@@ -2316,7 +2299,7 @@
         <v>82</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>76</v>
@@ -2343,7 +2326,7 @@
         <v>84</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>76</v>
@@ -2370,7 +2353,7 @@
         <v>86</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>76</v>
@@ -2397,7 +2380,7 @@
         <v>88</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>76</v>
@@ -2424,7 +2407,7 @@
         <v>90</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>91</v>
@@ -2451,7 +2434,7 @@
         <v>93</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>91</v>
@@ -2478,7 +2461,7 @@
         <v>95</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>59</v>
@@ -2502,10 +2485,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>97</v>
+        <v>328</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>276</v>
+        <v>330</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>9</v>
@@ -2516,8 +2499,8 @@
       <c r="F42" s="2">
         <v>107.53890199999999</v>
       </c>
-      <c r="G42" s="2" t="s">
-        <v>98</v>
+      <c r="G42" s="5" t="s">
+        <v>331</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>11</v>
@@ -2529,10 +2512,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>59</v>
@@ -2544,7 +2527,7 @@
         <v>107.5841879</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>11</v>
@@ -2556,13 +2539,13 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E44" s="2">
         <v>16.457834600000002</v>
@@ -2571,7 +2554,7 @@
         <v>107.5842155</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>11</v>
@@ -2583,10 +2566,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>9</v>
@@ -2598,7 +2581,7 @@
         <v>107.5898061</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>11</v>
@@ -2610,10 +2593,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>59</v>
@@ -2625,7 +2608,7 @@
         <v>107.59127290000001</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>11</v>
@@ -2637,10 +2620,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>9</v>
@@ -2652,7 +2635,7 @@
         <v>107.5887</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>11</v>
@@ -2664,10 +2647,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>59</v>
@@ -2679,7 +2662,7 @@
         <v>107.5812344</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>11</v>
@@ -2691,10 +2674,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>59</v>
@@ -2706,7 +2689,7 @@
         <v>107.5758125</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H49" s="2" t="s">
         <v>11</v>
@@ -2718,10 +2701,10 @@
         <v>49</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>59</v>
@@ -2733,7 +2716,7 @@
         <v>107.5666428</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H50" s="2" t="s">
         <v>11</v>
@@ -2745,10 +2728,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>59</v>
@@ -2760,7 +2743,7 @@
         <v>107.5924182</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H51" s="2" t="s">
         <v>11</v>
@@ -2772,10 +2755,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>59</v>
@@ -2787,7 +2770,7 @@
         <v>107.5885002</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H52" s="2" t="s">
         <v>11</v>
@@ -2799,10 +2782,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>59</v>
@@ -2814,7 +2797,7 @@
         <v>107.5997497</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H53" s="2" t="s">
         <v>11</v>
@@ -2826,10 +2809,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>59</v>
@@ -2841,7 +2824,7 @@
         <v>107.6040878</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>11</v>
@@ -2853,10 +2836,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>59</v>
@@ -2868,7 +2851,7 @@
         <v>107.6078971</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>11</v>
@@ -2880,10 +2863,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>59</v>
@@ -2895,7 +2878,7 @@
         <v>107.65366779999999</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="H56" s="2" t="s">
         <v>11</v>
@@ -2907,10 +2890,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>9</v>
@@ -2922,7 +2905,7 @@
         <v>107.5094706</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>11</v>
@@ -2934,10 +2917,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>9</v>
@@ -2949,7 +2932,7 @@
         <v>107.5780681</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H58" s="2" t="s">
         <v>11</v>
@@ -2961,10 +2944,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>9</v>
@@ -2976,7 +2959,7 @@
         <v>107.5914458</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>11</v>
@@ -2988,10 +2971,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>9</v>
@@ -3003,7 +2986,7 @@
         <v>107.5712089</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>11</v>
@@ -3015,22 +2998,22 @@
         <v>60</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="E61" s="2">
-        <v>16.471778</v>
+        <v>16.351575700000001</v>
       </c>
       <c r="F61" s="2">
-        <v>107.5782705</v>
+        <v>107.5882024</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>11</v>
@@ -3042,22 +3025,22 @@
         <v>61</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E62" s="2">
-        <v>16.351575700000001</v>
+        <v>16.539455100000001</v>
       </c>
       <c r="F62" s="2">
-        <v>107.5882024</v>
+        <v>107.4709349</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H62" s="2" t="s">
         <v>11</v>
@@ -3069,22 +3052,22 @@
         <v>62</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E63" s="2">
-        <v>16.539455100000001</v>
+        <v>16.453249799999998</v>
       </c>
       <c r="F63" s="2">
-        <v>107.4709349</v>
+        <v>107.56329409999999</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>11</v>
@@ -3096,22 +3079,22 @@
         <v>63</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E64" s="2">
-        <v>16.453249799999998</v>
+        <v>16.5217578</v>
       </c>
       <c r="F64" s="2">
-        <v>107.56329409999999</v>
+        <v>107.57747569999999</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>11</v>
@@ -3123,22 +3106,22 @@
         <v>64</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="D65" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E65" s="2">
-        <v>16.5217578</v>
+        <v>16.5582703</v>
       </c>
       <c r="F65" s="2">
-        <v>107.57747569999999</v>
+        <v>107.46912589999999</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="H65" s="2" t="s">
         <v>11</v>
@@ -3150,22 +3133,22 @@
         <v>65</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E66" s="2">
-        <v>16.5582703</v>
+        <v>16.498332099999999</v>
       </c>
       <c r="F66" s="2">
-        <v>107.46912589999999</v>
+        <v>107.5798678</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H66" s="2" t="s">
         <v>11</v>
@@ -3177,22 +3160,22 @@
         <v>66</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E67" s="2">
-        <v>16.498332099999999</v>
+        <v>16.5053321</v>
       </c>
       <c r="F67" s="2">
-        <v>107.5798678</v>
+        <v>107.5785503</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H67" s="2" t="s">
         <v>11</v>
@@ -3204,22 +3187,22 @@
         <v>67</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E68" s="2">
-        <v>16.5053321</v>
+        <v>16.507373300000001</v>
       </c>
       <c r="F68" s="2">
-        <v>107.5785503</v>
+        <v>107.63578459999999</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H68" s="2" t="s">
         <v>11</v>
@@ -3231,22 +3214,22 @@
         <v>68</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="E69" s="2">
-        <v>16.507373300000001</v>
+        <v>16.411297399999999</v>
       </c>
       <c r="F69" s="2">
-        <v>107.63578459999999</v>
+        <v>107.5738937</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H69" s="2" t="s">
         <v>11</v>
@@ -3258,22 +3241,22 @@
         <v>69</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="E70" s="2">
-        <v>16.411297399999999</v>
+        <v>16.462172800000001</v>
       </c>
       <c r="F70" s="2">
-        <v>107.5738937</v>
+        <v>107.57073629999999</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>11</v>
@@ -3285,22 +3268,22 @@
         <v>70</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E71" s="2">
-        <v>16.453250400000002</v>
+        <v>16.433186800000001</v>
       </c>
       <c r="F71" s="2">
-        <v>107.544583</v>
+        <v>107.56539979999999</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H71" s="2" t="s">
         <v>11</v>
@@ -3312,22 +3295,22 @@
         <v>71</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="E72" s="2">
-        <v>16.462172800000001</v>
+        <v>16.451093700000001</v>
       </c>
       <c r="F72" s="2">
-        <v>107.57073629999999</v>
+        <v>107.5931525</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>11</v>
@@ -3339,22 +3322,22 @@
         <v>72</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E73" s="2">
-        <v>16.433186800000001</v>
+        <v>16.4566552</v>
       </c>
       <c r="F73" s="2">
-        <v>107.56539979999999</v>
+        <v>107.58094629999999</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>11</v>
@@ -3366,22 +3349,22 @@
         <v>73</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="E74" s="2">
-        <v>16.451093700000001</v>
+        <v>16.457212599999998</v>
       </c>
       <c r="F74" s="2">
-        <v>107.5931525</v>
+        <v>107.5788716</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H74" s="2" t="s">
         <v>11</v>
@@ -3393,22 +3376,22 @@
         <v>74</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="E75" s="2">
-        <v>16.4566552</v>
+        <v>16.4669715</v>
       </c>
       <c r="F75" s="2">
-        <v>107.58094629999999</v>
+        <v>107.5895601</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>11</v>
@@ -3420,22 +3403,22 @@
         <v>75</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="E76" s="2">
-        <v>16.457212599999998</v>
+        <v>16.459246700000001</v>
       </c>
       <c r="F76" s="2">
-        <v>107.5788716</v>
+        <v>107.5822457</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="H76" s="2" t="s">
         <v>11</v>
@@ -3447,22 +3430,22 @@
         <v>76</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E77" s="2">
-        <v>16.4669715</v>
+        <v>16.467682400000001</v>
       </c>
       <c r="F77" s="2">
-        <v>107.5895601</v>
+        <v>107.57918340000001</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H77" s="2" t="s">
         <v>11</v>
@@ -3474,22 +3457,22 @@
         <v>77</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E78" s="2">
-        <v>16.459246700000001</v>
+        <v>16.470303600000001</v>
       </c>
       <c r="F78" s="2">
-        <v>107.5822457</v>
+        <v>107.57848389999999</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H78" s="2" t="s">
         <v>11</v>
@@ -3501,22 +3484,22 @@
         <v>78</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E79" s="2">
-        <v>16.467682400000001</v>
+        <v>16.467545900000001</v>
       </c>
       <c r="F79" s="2">
-        <v>107.57918340000001</v>
+        <v>107.57642869999999</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>11</v>
@@ -3528,22 +3511,22 @@
         <v>79</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E80" s="2">
-        <v>16.470303600000001</v>
+        <v>16.4699025</v>
       </c>
       <c r="F80" s="2">
-        <v>107.57848389999999</v>
+        <v>107.5803251</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H80" s="2" t="s">
         <v>11</v>
@@ -3555,22 +3538,22 @@
         <v>80</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E81" s="2">
-        <v>16.467545900000001</v>
+        <v>16.470199099999999</v>
       </c>
       <c r="F81" s="2">
-        <v>107.57642869999999</v>
+        <v>107.5800933</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H81" s="2" t="s">
         <v>11</v>
@@ -3582,22 +3565,22 @@
         <v>81</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E82" s="2">
-        <v>16.4699025</v>
+        <v>16.470616199999998</v>
       </c>
       <c r="F82" s="2">
-        <v>107.5803251</v>
+        <v>107.5797647</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H82" s="2" t="s">
         <v>11</v>
@@ -3609,22 +3592,22 @@
         <v>82</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E83" s="2">
-        <v>16.470199099999999</v>
+        <v>16.468891599999999</v>
       </c>
       <c r="F83" s="2">
-        <v>107.5800933</v>
+        <v>107.5754008</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H83" s="2" t="s">
         <v>11</v>
@@ -3636,22 +3619,22 @@
         <v>83</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E84" s="2">
-        <v>16.470616199999998</v>
+        <v>16.469718199999999</v>
       </c>
       <c r="F84" s="2">
-        <v>107.5797647</v>
+        <v>107.5746783</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H84" s="2" t="s">
         <v>11</v>
@@ -3663,22 +3646,22 @@
         <v>84</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="D85" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E85" s="2">
-        <v>16.468891599999999</v>
+        <v>16.4663574</v>
       </c>
       <c r="F85" s="2">
-        <v>107.5754008</v>
+        <v>107.5802462</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H85" s="2" t="s">
         <v>11</v>
@@ -3690,22 +3673,22 @@
         <v>85</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E86" s="2">
-        <v>16.469718199999999</v>
+        <v>16.468033299999998</v>
       </c>
       <c r="F86" s="2">
-        <v>107.5746783</v>
+        <v>107.58556849999999</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H86" s="2" t="s">
         <v>11</v>
@@ -3717,22 +3700,22 @@
         <v>86</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="E87" s="2">
-        <v>16.4663574</v>
+        <v>16.459624900000001</v>
       </c>
       <c r="F87" s="2">
-        <v>107.5802462</v>
+        <v>107.5811082</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H87" s="2" t="s">
         <v>11</v>
@@ -3744,22 +3727,22 @@
         <v>87</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="E88" s="2">
-        <v>16.468033299999998</v>
+        <v>16.466781699999999</v>
       </c>
       <c r="F88" s="2">
-        <v>107.58556849999999</v>
+        <v>107.6421227</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H88" s="2" t="s">
         <v>11</v>
@@ -3771,22 +3754,22 @@
         <v>88</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E89" s="2">
-        <v>16.459624900000001</v>
+        <v>16.471596000000002</v>
       </c>
       <c r="F89" s="2">
-        <v>107.5811082</v>
+        <v>107.5800406</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H89" s="2" t="s">
         <v>11</v>
@@ -3798,22 +3781,22 @@
         <v>89</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E90" s="2">
-        <v>16.466781699999999</v>
+        <v>16.470597699999999</v>
       </c>
       <c r="F90" s="2">
-        <v>107.6421227</v>
+        <v>107.5824866</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H90" s="2" t="s">
         <v>11</v>
@@ -3825,22 +3808,22 @@
         <v>90</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E91" s="2">
-        <v>16.471596000000002</v>
+        <v>16.468743400000001</v>
       </c>
       <c r="F91" s="2">
-        <v>107.5800406</v>
+        <v>107.5783867</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>197</v>
+        <v>329</v>
       </c>
       <c r="H91" s="2" t="s">
         <v>11</v>
@@ -3852,22 +3835,22 @@
         <v>91</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E92" s="2">
-        <v>16.470597699999999</v>
+        <v>16.468038</v>
       </c>
       <c r="F92" s="2">
-        <v>107.5824866</v>
+        <v>107.5750678</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H92" s="2" t="s">
         <v>11</v>
@@ -3879,22 +3862,22 @@
         <v>92</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E93" s="2">
-        <v>16.468743400000001</v>
+        <v>16.470085000000001</v>
       </c>
       <c r="F93" s="2">
-        <v>107.5783867</v>
+        <v>107.57521970000001</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H93" s="2" t="s">
         <v>11</v>
@@ -3906,22 +3889,22 @@
         <v>93</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="E94" s="2">
-        <v>16.468038</v>
+        <v>16.475617100000001</v>
       </c>
       <c r="F94" s="2">
-        <v>107.5750678</v>
+        <v>107.5806219</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H94" s="2" t="s">
         <v>11</v>
@@ -3933,22 +3916,22 @@
         <v>94</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="E95" s="2">
-        <v>16.470085000000001</v>
+        <v>16.471959300000002</v>
       </c>
       <c r="F95" s="2">
-        <v>107.57521970000001</v>
+        <v>107.583647</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H95" s="2" t="s">
         <v>11</v>
@@ -3960,22 +3943,22 @@
         <v>95</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E96" s="2">
-        <v>16.475617100000001</v>
+        <v>16.469853499999999</v>
       </c>
       <c r="F96" s="2">
-        <v>107.5806219</v>
+        <v>107.5825025</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H96" s="2" t="s">
         <v>11</v>
@@ -3987,22 +3970,22 @@
         <v>96</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E97" s="2">
-        <v>16.471959300000002</v>
+        <v>16.471307299999999</v>
       </c>
       <c r="F97" s="2">
-        <v>107.583647</v>
+        <v>107.5819424</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H97" s="2" t="s">
         <v>11</v>
@@ -4014,22 +3997,22 @@
         <v>97</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E98" s="2">
-        <v>16.469853499999999</v>
+        <v>16.472959299999999</v>
       </c>
       <c r="F98" s="2">
-        <v>107.5825025</v>
+        <v>107.58079309999999</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="H98" s="2" t="s">
         <v>11</v>
@@ -4041,22 +4024,22 @@
         <v>98</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="E99" s="2">
-        <v>16.471307299999999</v>
+        <v>16.4779515</v>
       </c>
       <c r="F99" s="2">
-        <v>107.5819424</v>
+        <v>107.5875648</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="H99" s="2" t="s">
         <v>11</v>
@@ -4068,22 +4051,22 @@
         <v>99</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="D100" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E100" s="2">
-        <v>16.472959299999999</v>
+        <v>16.452861200000001</v>
       </c>
       <c r="F100" s="2">
-        <v>107.58079309999999</v>
+        <v>107.58766319999999</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="H100" s="2" t="s">
         <v>11</v>
@@ -4095,81 +4078,29 @@
         <v>100</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="D101" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E101" s="2">
-        <v>16.4779515</v>
+        <v>16.4715813</v>
       </c>
       <c r="F101" s="2">
-        <v>107.5875648</v>
+        <v>107.5763379</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="H101" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="2">
-        <f t="shared" si="0"/>
-        <v>101</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="C102" s="4" t="s">
-        <v>336</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E102" s="2">
-        <v>16.452861200000001</v>
-      </c>
-      <c r="F102" s="2">
-        <v>107.58766319999999</v>
-      </c>
-      <c r="G102" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="H102" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="103" spans="1:8" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="2">
-        <f t="shared" si="0"/>
-        <v>102</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="C103" s="4" t="s">
-        <v>337</v>
-      </c>
-      <c r="D103" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E103" s="2">
-        <v>16.4715813</v>
-      </c>
-      <c r="F103" s="2">
-        <v>107.5763379</v>
-      </c>
-      <c r="G103" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="H103" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
+    <row r="102" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="103" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="104" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="105" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="106" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -5065,11 +4996,9 @@
     <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
-  <pageSetup orientation="landscape"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5083,21 +5012,21 @@
   <sheetData>
     <row r="1" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C2" s="2">
         <v>5</v>
@@ -5105,10 +5034,10 @@
     </row>
     <row r="3" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C3" s="2">
         <v>92</v>
@@ -5116,10 +5045,10 @@
     </row>
     <row r="4" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C4" s="2">
         <v>52</v>
@@ -5127,10 +5056,10 @@
     </row>
     <row r="5" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C5" s="2">
         <v>63</v>
@@ -5138,10 +5067,10 @@
     </row>
     <row r="6" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C6" s="2">
         <v>90</v>
@@ -5149,10 +5078,10 @@
     </row>
     <row r="7" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C7" s="2">
         <v>70</v>
@@ -5160,10 +5089,10 @@
     </row>
     <row r="8" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C8" s="2">
         <v>80</v>
@@ -5171,10 +5100,10 @@
     </row>
     <row r="9" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C9" s="2">
         <v>10</v>
@@ -5182,10 +5111,10 @@
     </row>
     <row r="10" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C10" s="2">
         <v>50</v>
@@ -5193,10 +5122,10 @@
     </row>
     <row r="11" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C11" s="2">
         <v>56</v>
@@ -5204,10 +5133,10 @@
     </row>
     <row r="12" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C12" s="2">
         <v>17</v>
@@ -5215,10 +5144,10 @@
     </row>
     <row r="13" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C13" s="2">
         <v>30</v>
@@ -5226,10 +5155,10 @@
     </row>
     <row r="14" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C14" s="2">
         <v>19</v>
@@ -5237,10 +5166,10 @@
     </row>
     <row r="15" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C15" s="2">
         <v>87</v>
@@ -5248,10 +5177,10 @@
     </row>
     <row r="16" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C16" s="2">
         <v>7</v>
@@ -5259,10 +5188,10 @@
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C17" s="2">
         <v>78</v>
@@ -5270,10 +5199,10 @@
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C18" s="2">
         <v>16</v>
@@ -5281,10 +5210,10 @@
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C19" s="2">
         <v>72</v>
@@ -5292,10 +5221,10 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C20" s="2">
         <v>92</v>
@@ -5303,10 +5232,10 @@
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C21" s="2">
         <v>54</v>
@@ -5314,10 +5243,10 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C22" s="2">
         <v>14</v>
@@ -5325,10 +5254,10 @@
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C23" s="2">
         <v>12</v>
@@ -5336,10 +5265,10 @@
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C24" s="2">
         <v>50</v>
@@ -5347,10 +5276,10 @@
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C25" s="2">
         <v>49</v>
@@ -5358,10 +5287,10 @@
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C26" s="2">
         <v>95</v>
@@ -5369,10 +5298,10 @@
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C27" s="2">
         <v>79</v>
@@ -5380,10 +5309,10 @@
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C28" s="2">
         <v>75</v>
@@ -5391,10 +5320,10 @@
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C29" s="2">
         <v>13</v>
@@ -5402,10 +5331,10 @@
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C30" s="2">
         <v>16</v>
@@ -5413,10 +5342,10 @@
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C31" s="2">
         <v>22</v>
@@ -5424,10 +5353,10 @@
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C32" s="2">
         <v>29</v>
@@ -5435,10 +5364,10 @@
     </row>
     <row r="33" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C33" s="2">
         <v>83</v>
@@ -5446,10 +5375,10 @@
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C34" s="2">
         <v>54</v>
@@ -5457,10 +5386,10 @@
     </row>
     <row r="35" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C35" s="2">
         <v>60</v>
@@ -5468,10 +5397,10 @@
     </row>
     <row r="36" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C36" s="2">
         <v>26</v>
@@ -5479,10 +5408,10 @@
     </row>
     <row r="37" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C37" s="2">
         <v>17</v>
@@ -5490,10 +5419,10 @@
     </row>
     <row r="38" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C38" s="2">
         <v>53</v>
@@ -5501,10 +5430,10 @@
     </row>
     <row r="39" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C39" s="2">
         <v>20</v>
@@ -5512,10 +5441,10 @@
     </row>
     <row r="40" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C40" s="2">
         <v>12</v>
@@ -5523,10 +5452,10 @@
     </row>
     <row r="41" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C41" s="2">
         <v>84</v>
@@ -5534,10 +5463,10 @@
     </row>
     <row r="42" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C42" s="2">
         <v>95</v>
@@ -5545,10 +5474,10 @@
     </row>
     <row r="43" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C43" s="2">
         <v>35</v>
@@ -5556,10 +5485,10 @@
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C44" s="2">
         <v>32</v>
@@ -5567,10 +5496,10 @@
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C45" s="2">
         <v>99</v>
@@ -5578,10 +5507,10 @@
     </row>
     <row r="46" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C46" s="2">
         <v>32</v>
@@ -5589,10 +5518,10 @@
     </row>
     <row r="47" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C47" s="2">
         <v>17</v>
@@ -5600,10 +5529,10 @@
     </row>
     <row r="48" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C48" s="2">
         <v>39</v>
@@ -5611,10 +5540,10 @@
     </row>
     <row r="49" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C49" s="2">
         <v>70</v>
@@ -5622,10 +5551,10 @@
     </row>
     <row r="50" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C50" s="2">
         <v>54</v>
@@ -5633,10 +5562,10 @@
     </row>
     <row r="51" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C51" s="2">
         <v>47</v>
@@ -5644,10 +5573,10 @@
     </row>
     <row r="52" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C52" s="2">
         <v>38</v>
@@ -5655,10 +5584,10 @@
     </row>
     <row r="53" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C53" s="2">
         <v>92</v>
@@ -5666,10 +5595,10 @@
     </row>
     <row r="54" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C54" s="2">
         <v>31</v>
@@ -5677,10 +5606,10 @@
     </row>
     <row r="55" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C55" s="2">
         <v>86</v>
@@ -5688,10 +5617,10 @@
     </row>
     <row r="56" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C56" s="2">
         <v>42</v>
@@ -5699,10 +5628,10 @@
     </row>
     <row r="57" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C57" s="2">
         <v>16</v>
@@ -5710,10 +5639,10 @@
     </row>
     <row r="58" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C58" s="2">
         <v>73</v>
@@ -5721,10 +5650,10 @@
     </row>
     <row r="59" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C59" s="2">
         <v>36</v>
@@ -5732,10 +5661,10 @@
     </row>
     <row r="60" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C60" s="2">
         <v>7</v>
@@ -5743,10 +5672,10 @@
     </row>
     <row r="61" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C61" s="2">
         <v>11</v>
@@ -5754,10 +5683,10 @@
     </row>
     <row r="62" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C62" s="2">
         <v>89</v>
@@ -5765,10 +5694,10 @@
     </row>
     <row r="63" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C63" s="2">
         <v>98</v>
@@ -5776,10 +5705,10 @@
     </row>
     <row r="64" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C64" s="2">
         <v>71</v>
@@ -5787,10 +5716,10 @@
     </row>
     <row r="65" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C65" s="2">
         <v>75</v>
@@ -5798,10 +5727,10 @@
     </row>
     <row r="66" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C66" s="2">
         <v>93</v>
@@ -5809,10 +5738,10 @@
     </row>
     <row r="67" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C67" s="2">
         <v>25</v>
@@ -5820,10 +5749,10 @@
     </row>
     <row r="68" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C68" s="2">
         <v>39</v>
@@ -5831,10 +5760,10 @@
     </row>
     <row r="69" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C69" s="2">
         <v>76</v>
@@ -5842,10 +5771,10 @@
     </row>
     <row r="70" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C70" s="2">
         <v>23</v>
@@ -5853,10 +5782,10 @@
     </row>
     <row r="71" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C71" s="2">
         <v>77</v>
@@ -5864,10 +5793,10 @@
     </row>
     <row r="72" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C72" s="2">
         <v>29</v>
@@ -5875,10 +5804,10 @@
     </row>
     <row r="73" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C73" s="2">
         <v>40</v>
@@ -5886,10 +5815,10 @@
     </row>
     <row r="74" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C74" s="2">
         <v>101</v>
@@ -5897,10 +5826,10 @@
     </row>
     <row r="75" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C75" s="2">
         <v>41</v>
@@ -5908,10 +5837,10 @@
     </row>
     <row r="76" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C76" s="2">
         <v>5</v>

</xml_diff>

<commit_message>
feat: Update AI Planner (Save Itinerary, Counter UI), RBAC security, Reset Password and Mobile Responsive UI
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Locations" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Users" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Likes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Locations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Likes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,42 +431,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>lat</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>lng</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>image</t>
         </is>
@@ -3387,7 +3399,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Tượng đài Phan Bội Châu là điểm đến lịch sử nổi bật, tôn vinh nhà yêu nước tại trung tâm thành phố Vinh, Nghệ An.</t>
+          <t>Khu lưu niệm Phan Bội Châu tại Huế là nơi cụ đã sống những năm tháng cuối đời (1925-1940), gắn liền với biệt danh 'Ông già Bến Ngự'. Nơi đây lưu giữ nhiều kỷ vật và là di tích lịch sử văn hóa cấp quốc gia.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4039,22 +4051,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>role</t>
         </is>
@@ -4475,17 +4487,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>user_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>user_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>location_name</t>
         </is>

</xml_diff>